<commit_message>
docs: bound text fields in data model
</commit_message>
<xml_diff>
--- a/docs/deliveries/2/data-catalog/academix-data-catalog.xlsx
+++ b/docs/deliveries/2/data-catalog/academix-data-catalog.xlsx
@@ -692,7 +692,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="39.75" customHeight="1" s="5">
+    <row r="3" ht="40" customHeight="1" s="5">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>institutions</t>
@@ -897,7 +897,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(254)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -912,7 +912,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Correo de referencia; unicidad se define con proveedor de identidad. Correo de referencia; límite, normalización y unicidad pendientes del proveedor de identidad.</t>
+          <t>Correo de referencia, máximo 254 caracteres; normalización y unicidad pendientes del contrato de autenticación.</t>
         </is>
       </c>
     </row>
@@ -1396,7 +1396,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="39.75" customHeight="1" s="5">
+    <row r="25" ht="40" customHeight="1" s="5">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>courses</t>
@@ -1620,7 +1620,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="39.75" customHeight="1" s="5">
+    <row r="32" ht="40" customHeight="1" s="5">
       <c r="A32" s="7" t="inlineStr">
         <is>
           <t>sections</t>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="39.75" customHeight="1" s="5">
+    <row r="38" ht="40" customHeight="1" s="5">
       <c r="A38" s="7" t="inlineStr">
         <is>
           <t>enrollments</t>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(16)</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -1840,7 +1840,7 @@
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>`teacher`, `assistant` o `student`. Dominio cerrado mediante CHECK: teacher, student, assistant.</t>
+          <t>Rol académico: teacher, assistant o student; máximo 16 caracteres y valores restringidos por CHECK.</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="39.75" customHeight="1" s="5">
+    <row r="45" ht="40" customHeight="1" s="5">
       <c r="A45" s="7" t="inlineStr">
         <is>
           <t>course_modules</t>
@@ -2228,7 +2228,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="39.75" customHeight="1" s="5">
+    <row r="51" ht="40" customHeight="1" s="5">
       <c r="A51" s="7" t="inlineStr">
         <is>
           <t>materials</t>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(16)</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>`markdown` o `file`. Dominio cerrado mediante CHECK: markdown, file.</t>
+          <t>Tipo de material: markdown o file; máximo 16 caracteres y valores restringidos por CHECK.</t>
         </is>
       </c>
     </row>
@@ -2288,11 +2288,11 @@
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Contenido textual cuando `kind = markdown`. Contenido textual de extensión variable; conservar text para Markdown o instrucciones.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="39.75" customHeight="1" s="5">
+          <t>Contenido Markdown de extensión variable; único campo text del modelo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="56" customHeight="1" s="5">
       <c r="A53" s="7" t="inlineStr">
         <is>
           <t>materials</t>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(1024)</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -2320,11 +2320,11 @@
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Clave interna para archivo externo futuro. Clave de extensión variable; proveedor y máximo pendientes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="39.75" customHeight="1" s="5">
+          <t>Clave interna del archivo externo, máximo 1024 caracteres; namespace por institución y validación en bytes según el proveedor futuro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="40" customHeight="1" s="5">
       <c r="A54" s="7" t="inlineStr">
         <is>
           <t>materials</t>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(255)</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
@@ -2352,11 +2352,11 @@
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>MIME del archivo futuro. Identificador MIME; lista permitida pendiente; no imponer tamaño arbitrario.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="39.75" customHeight="1" s="5">
+          <t>Tipo MIME del archivo, máximo 255 caracteres; lista de tipos permitidos pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="40" customHeight="1" s="5">
       <c r="A55" s="7" t="inlineStr">
         <is>
           <t>materials</t>
@@ -2612,7 +2612,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="39.75" customHeight="1" s="5">
+    <row r="63" ht="40" customHeight="1" s="5">
       <c r="A63" s="7" t="inlineStr">
         <is>
           <t>quizzes</t>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(10000)</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -2640,7 +2640,7 @@
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
-          <t>Instrucciones visibles. Contenido textual de extensión variable; conservar text para Markdown o instrucciones.</t>
+          <t>Instrucciones visibles, máximo 10000 caracteres para texto extenso de la evaluación.</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="39.75" customHeight="1" s="5">
+    <row r="66" ht="40" customHeight="1" s="5">
       <c r="A66" s="7" t="inlineStr">
         <is>
           <t>quizzes</t>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>Máximo de intentos por estudiante. Contenido textual de extensión variable; conservar text para Markdown o instrucciones.</t>
+          <t>Máximo de intentos por estudiante; integer positivo y NULL para intentos ilimitados.</t>
         </is>
       </c>
     </row>
@@ -2804,7 +2804,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="55.5" customHeight="1" s="5">
+    <row r="69" ht="56" customHeight="1" s="5">
       <c r="A69" s="7" t="inlineStr">
         <is>
           <t>quizzes</t>
@@ -3028,7 +3028,7 @@
         </is>
       </c>
     </row>
-    <row r="76" ht="39.75" customHeight="1" s="5">
+    <row r="76" ht="40" customHeight="1" s="5">
       <c r="A76" s="7" t="inlineStr">
         <is>
           <t>quiz_attempts</t>
@@ -3073,7 +3073,7 @@
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(16)</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="F77" s="7" t="inlineStr">
         <is>
-          <t>`in_progress`, `submitted`, `graded` o `cancelled`. Dominio cerrado mediante CHECK: in_progress, submitted, graded, cancelled.</t>
+          <t>Estado del intento: in_progress, submitted, graded o cancelled; máximo 16 caracteres y valores restringidos por CHECK.</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="39.75" customHeight="1" s="5">
+    <row r="81" ht="40" customHeight="1" s="5">
       <c r="A81" s="7" t="inlineStr">
         <is>
           <t>quiz_attempts</t>
@@ -3220,7 +3220,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="39.75" customHeight="1" s="5">
+    <row r="82" ht="40" customHeight="1" s="5">
       <c r="A82" s="7" t="inlineStr">
         <is>
           <t>quiz_attempts</t>
@@ -3252,7 +3252,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="39.75" customHeight="1" s="5">
+    <row r="83" ht="40" customHeight="1" s="5">
       <c r="A83" s="7" t="inlineStr">
         <is>
           <t>quiz_attempts</t>
@@ -3444,7 +3444,7 @@
         </is>
       </c>
     </row>
-    <row r="89" ht="39.75" customHeight="1" s="5">
+    <row r="89" ht="40" customHeight="1" s="5">
       <c r="A89" s="7" t="inlineStr">
         <is>
           <t>grade_items</t>
@@ -3732,7 +3732,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="39.75" customHeight="1" s="5">
+    <row r="98" ht="40" customHeight="1" s="5">
       <c r="A98" s="7" t="inlineStr">
         <is>
           <t>grades</t>
@@ -3764,7 +3764,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="39.75" customHeight="1" s="5">
+    <row r="99" ht="40" customHeight="1" s="5">
       <c r="A99" s="7" t="inlineStr">
         <is>
           <t>grades</t>
@@ -3988,7 +3988,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="39.75" customHeight="1" s="5">
+    <row r="106" ht="40" customHeight="1" s="5">
       <c r="A106" s="7" t="inlineStr">
         <is>
           <t>audit_events</t>
@@ -4001,7 +4001,7 @@
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(64)</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
@@ -4016,11 +4016,11 @@
       </c>
       <c r="F106" s="7" t="inlineStr">
         <is>
-          <t>Acción registrada. Vocabulario de acciones pendiente; longitud variable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="39.75" customHeight="1" s="5">
+          <t>Acción auditada, máximo 64 caracteres; vocabulario de acciones pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="40" customHeight="1" s="5">
       <c r="A107" s="7" t="inlineStr">
         <is>
           <t>audit_events</t>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>varchar(32)</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Tipo de recurso afectado. Vocabulario de recursos pendiente; longitud variable.</t>
+          <t>Tipo de recurso auditado, máximo 32 caracteres; vocabulario de recursos pendiente.</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4180,7 @@
         </is>
       </c>
     </row>
-    <row r="112" ht="55.5" customHeight="1" s="5">
+    <row r="112" ht="56" customHeight="1" s="5">
       <c r="A112" s="7" t="inlineStr">
         <is>
           <t>audit_events</t>

</xml_diff>